<commit_message>
feat: Trajectory Calculator (New IC) feat: Void Shield (New IC)
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla_Components_Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D587E7B-01B4-4442-98BC-1196C32F1812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89DFF1A-4AFA-4593-BDA2-6C45D750A638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
     <sheet name="BackpackFedWeapon" sheetId="3" r:id="rId2"/>
     <sheet name="ActiveProtectionSystem" sheetId="5" r:id="rId3"/>
+    <sheet name="TrajectoryCalculator" sheetId="6" r:id="rId4"/>
+    <sheet name="VoidShield" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="149">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -89,10 +91,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Desc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Supprot Contents</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -141,22 +139,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>To list all selectable projectiles</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>To select projectiles</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>To list all selectable friemodes</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>To select firemode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Indicates/set current firemode</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -191,10 +173,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>To list all slots projectiles come from</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Legacy</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -242,10 +220,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>To modify projectile spread</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Range</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -471,6 +445,147 @@
   </si>
   <si>
     <t>OnUse StatusEffects defined in the container will be triggered everytime the weapon shoots a projectile if true</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ShouldDrawTrajectory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TimeOfFly</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DrawColor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Color</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The max time of fly the projectile, only affect calculation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The color of the line</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whether should the calculator draw projectile trajectory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Color.Blue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Use a R,G,B,A in XML definition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Property Name</t>
+  </si>
+  <si>
+    <t>Property Type</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Support Contents</t>
+  </si>
+  <si>
+    <t>Default</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>Width of the rectangular collider in pixels</t>
+  </si>
+  <si>
+    <t>Ignored when Radius is above zero</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>Height of the rectangular collider in pixels</t>
+  </si>
+  <si>
+    <t>Radius</t>
+  </si>
+  <si>
+    <t>Radius of the circular collider in pixels</t>
+  </si>
+  <si>
+    <t>When above zero the collider is a circle and Width/Height are ignored</t>
+  </si>
+  <si>
+    <t>Offset</t>
+  </si>
+  <si>
+    <t>0,0</t>
+  </si>
+  <si>
+    <t>Visual</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Size used for the item's visibility extents, in pixels</t>
+  </si>
+  <si>
+    <t>Defaults to the sprite's own size when left at 0,0</t>
+  </si>
+  <si>
+    <t>AlwaysDraw</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>Draw the sprite even when the item is stowed in a container that does not draw its contents</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>Sprite</t>
+  </si>
+  <si>
+    <t>Offset of the collider and the sprite from the center of the item</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sprite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The sprite the component draws</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Will be affected by IsActive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Collider</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Use IsActive to engage/disengage Collider</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -502,7 +617,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -642,11 +757,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -707,32 +835,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1014,21 +1148,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EA240FE-1117-4C1F-984C-6020AD1A5D75}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.25" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.58203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="49.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.6640625" style="1"/>
+    <col min="5" max="5" width="44.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>10</v>
       </c>
@@ -1041,302 +1174,264 @@
       <c r="D1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>15</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="G1" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="31" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="31"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="32"/>
       <c r="B3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="32"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="33"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="4">
+        <v>28</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4">
         <v>0</v>
       </c>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="30" t="s">
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="31" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H5" s="3"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="31"/>
+      <c r="F5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="32"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="31"/>
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="32"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="4">
+      <c r="F7" s="4">
         <v>0</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="31"/>
+      <c r="G7" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="32"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="4">
+      <c r="F8" s="4">
         <v>0</v>
       </c>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="32"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="4" t="b">
+      <c r="F9" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="30" t="s">
-        <v>36</v>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="31" t="s">
+        <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G10" s="2" t="b">
+        <v>30</v>
+      </c>
+      <c r="F10" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H10" s="8"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="33"/>
       <c r="B11" s="5" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="5">
+        <v>7</v>
+      </c>
+      <c r="F11" s="1">
         <v>0</v>
       </c>
-      <c r="H11" s="10"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G11" s="10"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>7</v>
+      <c r="F12" s="26" t="s">
+        <v>45</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
       <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -1344,9 +1439,8 @@
       <c r="E18" s="11"/>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -1354,9 +1448,8 @@
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -1364,15 +1457,14 @@
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A9"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1410,88 +1502,88 @@
         <v>14</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="7" t="s">
-        <v>17</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="32"/>
+      <c r="B3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="32"/>
+      <c r="B4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="25"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="32"/>
+      <c r="B5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="31"/>
-      <c r="B3" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="31"/>
-      <c r="B4" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="25"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="31"/>
-      <c r="B5" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>7</v>
@@ -1500,19 +1592,19 @@
         <v>0</v>
       </c>
       <c r="G5" s="25" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
+      <c r="A6" s="33"/>
       <c r="B6" s="5" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>7</v>
@@ -1521,40 +1613,40 @@
         <v>1</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="31" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="31"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>7</v>
@@ -1565,15 +1657,15 @@
       <c r="G8" s="25"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="31"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>7</v>
@@ -1582,19 +1674,19 @@
         <v>0</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="31"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>7</v>
@@ -1605,15 +1697,15 @@
       <c r="G10" s="25"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="31"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>7</v>
@@ -1624,20 +1716,20 @@
       <c r="G11" s="25"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="30" t="s">
-        <v>36</v>
+      <c r="A12" s="31" t="s">
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F12" s="2" t="b">
         <v>1</v>
@@ -1645,69 +1737,69 @@
       <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="31"/>
-      <c r="B13" s="34" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="34" t="s">
+      <c r="A13" s="32"/>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="25"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="33"/>
+      <c r="B14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="34">
-        <v>0</v>
-      </c>
-      <c r="G13" s="25"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
-      <c r="B14" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>22</v>
-      </c>
       <c r="D14" s="5" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="b">
         <v>1</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>7</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B19" s="24"/>
       <c r="C19" s="24"/>
@@ -1717,11 +1809,11 @@
       <c r="G19" s="24"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="33"/>
-      <c r="C20" s="33"/>
+      <c r="A20" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
@@ -1796,27 +1888,27 @@
         <v>14</v>
       </c>
       <c r="E1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>17</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
-        <v>86</v>
+      <c r="A2" s="28" t="s">
+        <v>79</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E2" s="21" t="s">
         <v>7</v>
@@ -1827,15 +1919,15 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
+      <c r="A3" s="36"/>
       <c r="B3" s="14" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>7</v>
@@ -1844,19 +1936,19 @@
         <v>1</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
+      <c r="A4" s="36"/>
       <c r="B4" s="14" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>7</v>
@@ -1867,15 +1959,15 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
+      <c r="A5" s="36"/>
       <c r="B5" s="14" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" t="s">
         <v>66</v>
-      </c>
-      <c r="D5" t="s">
-        <v>73</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>7</v>
@@ -1886,15 +1978,15 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="28"/>
+      <c r="A6" s="36"/>
       <c r="B6" s="14" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>7</v>
@@ -1905,15 +1997,15 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="28"/>
+      <c r="A7" s="36"/>
       <c r="B7" s="14" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>7</v>
@@ -1924,15 +2016,15 @@
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="28"/>
+      <c r="A8" s="36"/>
       <c r="B8" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
         <v>59</v>
       </c>
-      <c r="C8" t="s">
-        <v>66</v>
-      </c>
       <c r="D8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>7</v>
@@ -1943,57 +2035,57 @@
       <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="28"/>
+      <c r="A9" s="36"/>
       <c r="B9" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="36"/>
+      <c r="B10" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="36"/>
+      <c r="B11" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
         <v>62</v>
       </c>
-      <c r="C9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="28"/>
-      <c r="B10" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="28"/>
-      <c r="B11" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" t="s">
-        <v>69</v>
-      </c>
       <c r="D11" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="E11" s="22" t="s">
         <v>7</v>
@@ -2004,15 +2096,15 @@
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
+      <c r="A12" s="36"/>
       <c r="B12" s="14" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E12" s="22" t="s">
         <v>7</v>
@@ -2023,15 +2115,15 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="28"/>
+      <c r="A13" s="36"/>
       <c r="B13" s="14" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E13" s="22" t="s">
         <v>7</v>
@@ -2042,15 +2134,15 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="28"/>
+      <c r="A14" s="36"/>
       <c r="B14" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E14" s="22" t="s">
         <v>7</v>
@@ -2061,15 +2153,15 @@
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
+      <c r="A15" s="37"/>
       <c r="B15" s="15" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>7</v>
@@ -2078,7 +2170,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -2090,29 +2182,29 @@
       <c r="F17" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
+      <c r="A19" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
+      <c r="A20" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
+      <c r="A21" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2124,4 +2216,331 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EFEE3F3-AD46-4780-8954-A48E858F415B}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.9140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.4140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="36"/>
+      <c r="B3" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1</v>
+      </c>
+      <c r="G3" s="25"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="37"/>
+      <c r="B4" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A4"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.25" customWidth="1"/>
+    <col min="4" max="4" width="84.08203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5" customWidth="1"/>
+    <col min="6" max="6" width="6.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="59.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="29"/>
+      <c r="B3" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="29"/>
+      <c r="B4" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="30"/>
+      <c r="B5" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="G5" s="27"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="28" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="29"/>
+      <c r="B7" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="30"/>
+      <c r="B8" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="35"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed VoidShield malfunction Fixed TrajectoryCalculator deviation in large steps
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla_Components_Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89DFF1A-4AFA-4593-BDA2-6C45D750A638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075AE46C-6BC1-41D2-9FCB-106512E1B17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="151">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -585,7 +585,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Use IsActive to engage/disengage Collider</t>
+    <t>StatusControl</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ShieldActive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whether the shield collider is enabled</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -617,7 +625,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -770,11 +778,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -844,6 +863,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -856,18 +881,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1185,7 +1214,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1208,7 +1237,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="32"/>
+      <c r="A3" s="34"/>
       <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
@@ -1229,7 +1258,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="33"/>
+      <c r="A4" s="35"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1248,7 +1277,7 @@
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="33" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1269,7 +1298,7 @@
       <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1288,7 +1317,7 @@
       <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
+      <c r="A7" s="34"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1309,7 +1338,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="32"/>
+      <c r="A8" s="34"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1328,7 +1357,7 @@
       <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="32"/>
+      <c r="A9" s="34"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1347,7 +1376,7 @@
       <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="33" t="s">
         <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1368,7 +1397,7 @@
       <c r="G10" s="8"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="33"/>
+      <c r="A11" s="35"/>
       <c r="B11" s="5" t="s">
         <v>46</v>
       </c>
@@ -1410,22 +1439,22 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="36"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1512,7 +1541,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1535,7 +1564,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="32"/>
+      <c r="A3" s="34"/>
       <c r="B3" s="1" t="s">
         <v>99</v>
       </c>
@@ -1556,7 +1585,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="32"/>
+      <c r="A4" s="34"/>
       <c r="B4" s="1" t="s">
         <v>88</v>
       </c>
@@ -1575,7 +1604,7 @@
       <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="32"/>
+      <c r="A5" s="34"/>
       <c r="B5" s="1" t="s">
         <v>90</v>
       </c>
@@ -1596,7 +1625,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="33"/>
+      <c r="A6" s="35"/>
       <c r="B6" s="5" t="s">
         <v>91</v>
       </c>
@@ -1617,7 +1646,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="33" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1638,7 +1667,7 @@
       <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="32"/>
+      <c r="A8" s="34"/>
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1657,7 +1686,7 @@
       <c r="G8" s="25"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="32"/>
+      <c r="A9" s="34"/>
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1678,7 +1707,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="32"/>
+      <c r="A10" s="34"/>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1697,7 +1726,7 @@
       <c r="G10" s="25"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
+      <c r="A11" s="34"/>
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1716,7 +1745,7 @@
       <c r="G11" s="25"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="33" t="s">
         <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -1737,7 +1766,7 @@
       <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="32"/>
+      <c r="A13" s="34"/>
       <c r="B13" s="1" t="s">
         <v>46</v>
       </c>
@@ -1756,7 +1785,7 @@
       <c r="G13" s="25"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="33"/>
+      <c r="A14" s="35"/>
       <c r="B14" s="5" t="s">
         <v>104</v>
       </c>
@@ -1809,11 +1838,11 @@
       <c r="G19" s="24"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
@@ -1919,7 +1948,7 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="36"/>
+      <c r="A3" s="37"/>
       <c r="B3" s="14" t="s">
         <v>49</v>
       </c>
@@ -1940,7 +1969,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="36"/>
+      <c r="A4" s="37"/>
       <c r="B4" s="14" t="s">
         <v>50</v>
       </c>
@@ -1959,7 +1988,7 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="36"/>
+      <c r="A5" s="37"/>
       <c r="B5" s="14" t="s">
         <v>51</v>
       </c>
@@ -1978,7 +2007,7 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="36"/>
+      <c r="A6" s="37"/>
       <c r="B6" s="14" t="s">
         <v>53</v>
       </c>
@@ -1997,7 +2026,7 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="36"/>
+      <c r="A7" s="37"/>
       <c r="B7" s="14" t="s">
         <v>86</v>
       </c>
@@ -2016,7 +2045,7 @@
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="36"/>
+      <c r="A8" s="37"/>
       <c r="B8" s="14" t="s">
         <v>52</v>
       </c>
@@ -2035,7 +2064,7 @@
       <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="36"/>
+      <c r="A9" s="37"/>
       <c r="B9" s="14" t="s">
         <v>55</v>
       </c>
@@ -2056,7 +2085,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="36"/>
+      <c r="A10" s="37"/>
       <c r="B10" s="14" t="s">
         <v>54</v>
       </c>
@@ -2077,7 +2106,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="36"/>
+      <c r="A11" s="37"/>
       <c r="B11" s="14" t="s">
         <v>56</v>
       </c>
@@ -2096,7 +2125,7 @@
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="36"/>
+      <c r="A12" s="37"/>
       <c r="B12" s="14" t="s">
         <v>57</v>
       </c>
@@ -2115,7 +2144,7 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="36"/>
+      <c r="A13" s="37"/>
       <c r="B13" s="14" t="s">
         <v>58</v>
       </c>
@@ -2134,7 +2163,7 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="36"/>
+      <c r="A14" s="37"/>
       <c r="B14" s="14" t="s">
         <v>81</v>
       </c>
@@ -2153,7 +2182,7 @@
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="37"/>
+      <c r="A15" s="38"/>
       <c r="B15" s="15" t="s">
         <v>82</v>
       </c>
@@ -2182,29 +2211,29 @@
       <c r="F17" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="35" t="s">
+      <c r="A20" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2278,7 +2307,7 @@
       <c r="G2" s="8"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="36"/>
+      <c r="A3" s="37"/>
       <c r="B3" s="1" t="s">
         <v>108</v>
       </c>
@@ -2297,7 +2326,7 @@
       <c r="G3" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="37"/>
+      <c r="A4" s="38"/>
       <c r="B4" s="5" t="s">
         <v>109</v>
       </c>
@@ -2332,7 +2361,7 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.25" customWidth="1"/>
     <col min="4" max="4" width="84.08203125" bestFit="1" customWidth="1"/>
@@ -2511,27 +2540,46 @@
       </c>
       <c r="G8" s="10"/>
     </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>149</v>
+      </c>
+      <c r="C9" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" s="39" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="41" t="s">
+        <v>7</v>
+      </c>
+    </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
+      <c r="A13" s="31"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="38" t="s">
-        <v>148</v>
-      </c>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="38"/>
+      <c r="A14" s="32"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Removed Size from VoidShield Fixed Patch not working for VoidShield Now Sprite element using its own depth rather than item depth Updated Doc
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla_Components_Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075AE46C-6BC1-41D2-9FCB-106512E1B17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9754EFFA-8469-4E13-99D2-FA660A4CADE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="150">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -538,62 +538,62 @@
     <t>0,0</t>
   </si>
   <si>
+    <t>AlwaysDraw</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>Draw the sprite even when the item is stowed in a container that does not draw its contents</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>Sprite</t>
+  </si>
+  <si>
+    <t>Offset of the collider and the sprite from the center of the item</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sprite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The sprite the component draws</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Collider</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusControl</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ShieldActive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whether the shield collider is enabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USE A FULL &lt;Sprite/&gt;ELEMENT HERE!!!!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>Visual</t>
-  </si>
-  <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>Size used for the item's visibility extents, in pixels</t>
-  </si>
-  <si>
-    <t>Defaults to the sprite's own size when left at 0,0</t>
-  </si>
-  <si>
-    <t>AlwaysDraw</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>Draw the sprite even when the item is stowed in a container that does not draw its contents</t>
-  </si>
-  <si>
-    <t>TRUE</t>
-  </si>
-  <si>
-    <t>Sprite</t>
-  </si>
-  <si>
-    <t>Offset of the collider and the sprite from the center of the item</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Sprite</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The sprite the component draws</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Will be affected by IsActive</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Collider</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>StatusControl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ShieldActive</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Whether the shield collider is enabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USE AT YOUR OWN RISK NOT IMPL YET</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Will be affected by ShieldActive</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -793,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -857,46 +857,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1214,7 +1210,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1237,7 +1233,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="34"/>
+      <c r="A3" s="33"/>
       <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
@@ -1258,7 +1254,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="35"/>
+      <c r="A4" s="34"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1277,7 +1273,7 @@
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="32" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1298,7 +1294,7 @@
       <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="34"/>
+      <c r="A6" s="33"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1317,7 +1313,7 @@
       <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="34"/>
+      <c r="A7" s="33"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1338,7 +1334,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="34"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1357,7 +1353,7 @@
       <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="34"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1376,7 +1372,7 @@
       <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="32" t="s">
         <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1397,7 +1393,7 @@
       <c r="G10" s="8"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="35"/>
+      <c r="A11" s="34"/>
       <c r="B11" s="5" t="s">
         <v>46</v>
       </c>
@@ -1439,22 +1435,22 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="36"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1541,7 +1537,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1564,7 +1560,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="34"/>
+      <c r="A3" s="33"/>
       <c r="B3" s="1" t="s">
         <v>99</v>
       </c>
@@ -1585,7 +1581,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="34"/>
+      <c r="A4" s="33"/>
       <c r="B4" s="1" t="s">
         <v>88</v>
       </c>
@@ -1604,7 +1600,7 @@
       <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="34"/>
+      <c r="A5" s="33"/>
       <c r="B5" s="1" t="s">
         <v>90</v>
       </c>
@@ -1625,7 +1621,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="35"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="5" t="s">
         <v>91</v>
       </c>
@@ -1646,7 +1642,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="32" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1667,7 +1663,7 @@
       <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="34"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1686,7 +1682,7 @@
       <c r="G8" s="25"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="34"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1707,7 +1703,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="34"/>
+      <c r="A10" s="33"/>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1726,7 +1722,7 @@
       <c r="G10" s="25"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="34"/>
+      <c r="A11" s="33"/>
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1745,7 +1741,7 @@
       <c r="G11" s="25"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="32" t="s">
         <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -1766,7 +1762,7 @@
       <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="34"/>
+      <c r="A13" s="33"/>
       <c r="B13" s="1" t="s">
         <v>46</v>
       </c>
@@ -1785,7 +1781,7 @@
       <c r="G13" s="25"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="35"/>
+      <c r="A14" s="34"/>
       <c r="B14" s="5" t="s">
         <v>104</v>
       </c>
@@ -1838,11 +1834,11 @@
       <c r="G19" s="24"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
@@ -1927,7 +1923,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>79</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -1948,7 +1944,7 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="37"/>
+      <c r="A3" s="30"/>
       <c r="B3" s="14" t="s">
         <v>49</v>
       </c>
@@ -1969,7 +1965,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="37"/>
+      <c r="A4" s="30"/>
       <c r="B4" s="14" t="s">
         <v>50</v>
       </c>
@@ -1988,7 +1984,7 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="37"/>
+      <c r="A5" s="30"/>
       <c r="B5" s="14" t="s">
         <v>51</v>
       </c>
@@ -2007,7 +2003,7 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="37"/>
+      <c r="A6" s="30"/>
       <c r="B6" s="14" t="s">
         <v>53</v>
       </c>
@@ -2026,7 +2022,7 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="37"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="14" t="s">
         <v>86</v>
       </c>
@@ -2045,7 +2041,7 @@
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="37"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="14" t="s">
         <v>52</v>
       </c>
@@ -2064,7 +2060,7 @@
       <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="37"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="14" t="s">
         <v>55</v>
       </c>
@@ -2085,7 +2081,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="37"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="14" t="s">
         <v>54</v>
       </c>
@@ -2106,7 +2102,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="37"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="14" t="s">
         <v>56</v>
       </c>
@@ -2125,7 +2121,7 @@
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="37"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="14" t="s">
         <v>57</v>
       </c>
@@ -2144,7 +2140,7 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="37"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="14" t="s">
         <v>58</v>
       </c>
@@ -2163,7 +2159,7 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="37"/>
+      <c r="A14" s="30"/>
       <c r="B14" s="14" t="s">
         <v>81</v>
       </c>
@@ -2182,7 +2178,7 @@
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="38"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="15" t="s">
         <v>82</v>
       </c>
@@ -2211,29 +2207,29 @@
       <c r="F17" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2286,7 +2282,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -2307,7 +2303,7 @@
       <c r="G2" s="8"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="37"/>
+      <c r="A3" s="30"/>
       <c r="B3" s="1" t="s">
         <v>108</v>
       </c>
@@ -2326,7 +2322,7 @@
       <c r="G3" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="38"/>
+      <c r="A4" s="31"/>
       <c r="B4" s="5" t="s">
         <v>109</v>
       </c>
@@ -2358,7 +2354,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -2394,8 +2390,8 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
-        <v>147</v>
+      <c r="A2" s="29" t="s">
+        <v>142</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>123</v>
@@ -2417,7 +2413,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
+      <c r="A3" s="37"/>
       <c r="B3" s="1" t="s">
         <v>127</v>
       </c>
@@ -2438,7 +2434,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="29"/>
+      <c r="A4" s="37"/>
       <c r="B4" s="1" t="s">
         <v>129</v>
       </c>
@@ -2459,7 +2455,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="30"/>
+      <c r="A5" s="38"/>
       <c r="B5" s="5" t="s">
         <v>132</v>
       </c>
@@ -2467,7 +2463,7 @@
         <v>60</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>30</v>
@@ -2475,118 +2471,101 @@
       <c r="F5" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="G5" s="27"/>
+      <c r="G5" s="40" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="G6" s="8" t="s">
+      <c r="F6" s="4" t="s">
         <v>137</v>
       </c>
+      <c r="G6" s="25" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="1" t="s">
+      <c r="A7" s="31"/>
+      <c r="B7" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="C7" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="D7" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="G7" s="25" t="s">
+      <c r="F7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="30"/>
-      <c r="B8" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="A8" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G8" s="10"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="42" t="s">
-        <v>148</v>
-      </c>
-      <c r="B9" s="39" t="s">
-        <v>149</v>
-      </c>
-      <c r="C9" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="39" t="s">
-        <v>150</v>
-      </c>
-      <c r="E9" s="39" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="40" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="41" t="s">
-        <v>7</v>
-      </c>
+      <c r="E8" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="36"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="31"/>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
+      <c r="A13" s="39"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:G14"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>